<commit_message>
evaluation: complete final RAG evaluation
</commit_message>
<xml_diff>
--- a/eval/day1_results(rerank-v3).xlsx
+++ b/eval/day1_results(rerank-v3).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ragflow-maxkb-support\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF5F75A-AF67-43F2-83B7-BE99ADA69606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFD8CC5-476D-4562-AD0E-9B33797279C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6990" yWindow="5590" windowWidth="25710" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4180" yWindow="4180" windowWidth="32150" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>